<commit_message>
Don't need to care previous roster's ward requirement
Don't need to care previous roster's ward requirement
</commit_message>
<xml_diff>
--- a/test/production/20260209-20260308/result.xlsx
+++ b/test/production/20260209-20260308/result.xlsx
@@ -246,12 +246,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="5"/>
+        <bgColor indexed="5"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="5">
@@ -306,7 +312,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
@@ -329,6 +335,9 @@
     <xf fontId="4" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf fontId="3" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf fontId="2" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
+    <xf fontId="3" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="0" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2692,25 +2701,25 @@
       <c r="J17" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="K17" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="L17" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="M17" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="N17" s="8" t="s">
+      <c r="K17" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="L17" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="M17" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N17" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="O17" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="P17" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q17" t="s">
+      <c r="O17" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="P17" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q17" s="22" t="s">
         <v>40</v>
       </c>
       <c r="R17" t="s">

</xml_diff>